<commit_message>
Regenerate manuscript example outputs
</commit_message>
<xml_diff>
--- a/examples/1JNJ/InterfaceScout_1JNJ_all_results.xlsx
+++ b/examples/1JNJ/InterfaceScout_1JNJ_all_results.xlsx
@@ -14,7 +14,7 @@
     <sheet name="Patch_Members" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Run_Method'!$A$1:$B$47</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Run_Method'!$A$1:$B$45</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Map_Definitions'!$A$1:$F$12</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Residue_Values'!$A$1:$O$83</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Patches'!$A$1:$R$146</definedName>
@@ -423,7 +423,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B47"/>
+  <dimension ref="A1:B45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -709,107 +709,105 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>method.parameter_selection.selection_workflow_run</t>
-        </is>
-      </c>
-      <c r="B26" t="n">
-        <v>34329264963</v>
+          <t>method.parameter_selection.uses_experimental_adsorption_labels</t>
+        </is>
+      </c>
+      <c r="B26" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>method.parameter_selection.selection_commit</t>
-        </is>
-      </c>
-      <c r="B27" t="inlineStr">
-        <is>
-          <t>ba0e63b7b82a222856ff75a6dd39409b89b664dd</t>
-        </is>
+          <t>method.patch_radius_A</t>
+        </is>
+      </c>
+      <c r="B27" t="n">
+        <v>8</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>method.parameter_selection.uses_experimental_adsorption_labels</t>
-        </is>
-      </c>
-      <c r="B28" t="b">
-        <v>0</v>
+          <t>method.patch_definition</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>non-transitive local surface neighbourhood around a chemistry-patch maximum</t>
+        </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>method.patch_radius_A</t>
-        </is>
-      </c>
-      <c r="B29" t="n">
-        <v>8</v>
+          <t>method.orientation</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>coarse outward C-alpha face consistency</t>
+        </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>method.patch_definition</t>
+          <t>method.ranking</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>non-transitive local surface neighbourhood around a chemistry-patch maximum</t>
+          <t>Pareto fronts across chemistry support, accessibility, patch coherence and orientation coherence; no weighted sum</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>method.orientation</t>
-        </is>
-      </c>
-      <c r="B31" t="inlineStr">
-        <is>
-          <t>coarse outward C-alpha face consistency</t>
-        </is>
+          <t>method.single_pass_all_maps</t>
+        </is>
+      </c>
+      <c r="B31" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>method.ranking</t>
+          <t>scope.prediction_unit</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Pareto fronts across chemistry support, accessibility, patch coherence and orientation coherence; no weighted sum</t>
+          <t>coarse protein surface region / interface patch</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>method.single_pass_all_maps</t>
+          <t>scope.predicts_absolute_adsorption_free_energy</t>
         </is>
       </c>
       <c r="B33" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>scope.prediction_unit</t>
-        </is>
-      </c>
-      <c r="B34" t="inlineStr">
-        <is>
-          <t>coarse protein surface region / interface patch</t>
-        </is>
+          <t>scope.predicts_adsorption_amount</t>
+        </is>
+      </c>
+      <c r="B34" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>scope.predicts_absolute_adsorption_free_energy</t>
+          <t>scope.predicts_unique_orientation</t>
         </is>
       </c>
       <c r="B35" t="b">
@@ -819,7 +817,7 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>scope.predicts_adsorption_amount</t>
+          <t>scope.models_adsorption_induced_unfolding</t>
         </is>
       </c>
       <c r="B36" t="b">
@@ -829,7 +827,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>scope.predicts_unique_orientation</t>
+          <t>scope.benchmark_fitted_weights</t>
         </is>
       </c>
       <c r="B37" t="b">
@@ -839,7 +837,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>scope.models_adsorption_induced_unfolding</t>
+          <t>scope.residue_precision_claim</t>
         </is>
       </c>
       <c r="B38" t="b">
@@ -849,61 +847,63 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>scope.benchmark_fitted_weights</t>
-        </is>
-      </c>
-      <c r="B39" t="b">
-        <v>0</v>
+          <t>diagnostics.n_surface_residues</t>
+        </is>
+      </c>
+      <c r="B39" t="n">
+        <v>85</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>scope.residue_precision_claim</t>
-        </is>
-      </c>
-      <c r="B40" t="b">
-        <v>0</v>
+          <t>diagnostics.surface_residue_keys</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>A:0:; A:1:; A:2:; A:3:; A:4:; A:6:; A:7:; A:8:; A:10:; A:11:; A:12:; A:13:; A:14:; A:15:; A:16:; A:17:; A:18:; A:19:; A:20:; A:22:; A:24:; A:26:; A:28:; A:29:; A:31:; A:32:; A:33:; A:34:; A:36:; A:38:; A:40:; A:41:; A:42:; A:43:; A:44:; A:45:; A:46:; A:47:; A:48:; A:49:; A:50:; A:51:; A:52:; A:53:; A:54:; A:55:; A:56:; A:57:; A:58:; A:59:; A:60:; A:61:; A:62:; A:63:; A:64:; A:65:; A:66:; A:67:; A:69:; A:71:; A:72:; A:73:; A:74:; A:75:; A:76:; A:77:; A:78:; A:79:; A:81:; A:83:; A:85:; A:86:; A:87:; A:88:; A:89:; A:90:; A:91:; A:92:; A:93:; A:94:; A:95:; A:96:; A:97:; A:98:; A:99:</t>
+        </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>diagnostics.n_surface_residues</t>
-        </is>
-      </c>
-      <c r="B41" t="n">
-        <v>85</v>
+          <t>composite_policy.type</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>derived_overlay</t>
+        </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>diagnostics.surface_residue_keys</t>
-        </is>
-      </c>
-      <c r="B42" t="inlineStr">
-        <is>
-          <t>A:0:; A:1:; A:2:; A:3:; A:4:; A:6:; A:7:; A:8:; A:10:; A:11:; A:12:; A:13:; A:14:; A:15:; A:16:; A:17:; A:18:; A:19:; A:20:; A:22:; A:24:; A:26:; A:28:; A:29:; A:31:; A:32:; A:33:; A:34:; A:36:; A:38:; A:40:; A:41:; A:42:; A:43:; A:44:; A:45:; A:46:; A:47:; A:48:; A:49:; A:50:; A:51:; A:52:; A:53:; A:54:; A:55:; A:56:; A:57:; A:58:; A:59:; A:60:; A:61:; A:62:; A:63:; A:64:; A:65:; A:66:; A:67:; A:69:; A:71:; A:72:; A:73:; A:74:; A:75:; A:76:; A:77:; A:78:; A:79:; A:81:; A:83:; A:85:; A:86:; A:87:; A:88:; A:89:; A:90:; A:91:; A:92:; A:93:; A:94:; A:95:; A:96:; A:97:; A:98:; A:99:</t>
-        </is>
+          <t>composite_policy.validated_as_combined_model</t>
+        </is>
+      </c>
+      <c r="B42" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>composite_policy.type</t>
+          <t>composite_policy.default_residue_rule</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>derived_overlay</t>
+          <t>maximum normalized support across selected canonical chemistry maps</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>composite_policy.validated_as_combined_model</t>
+          <t>composite_policy.double_counting</t>
         </is>
       </c>
       <c r="B44" t="b">
@@ -913,39 +913,17 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>composite_policy.default_residue_rule</t>
+          <t>composite_policy.weights</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>maximum normalized support across selected canonical chemistry maps</t>
-        </is>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" t="inlineStr">
-        <is>
-          <t>composite_policy.double_counting</t>
-        </is>
-      </c>
-      <c r="B46" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" t="inlineStr">
-        <is>
-          <t>composite_policy.weights</t>
-        </is>
-      </c>
-      <c r="B47" t="inlineStr">
-        <is>
           <t>none unless externally known surface composition is supplied in a future explicit model extension</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:B47"/>
+  <autoFilter ref="A1:B45"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1180,7 +1158,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Oxide-like surface chemistry represented by the frozen carboxylate-compatible oxide channel.</t>
+          <t>Oxide-like surface chemistry represented by the carboxylate-compatible oxide channel.</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -3991,7 +3969,7 @@
         <v>0.81951</v>
       </c>
       <c r="P2" t="n">
-        <v>0.972165506193017</v>
+        <v>0.9721655061930171</v>
       </c>
       <c r="Q2" t="inlineStr">
         <is>
@@ -4341,7 +4319,7 @@
         <v>0.5047999999999999</v>
       </c>
       <c r="P7" t="n">
-        <v>0.9405288652176459</v>
+        <v>0.940528865217646</v>
       </c>
       <c r="Q7" t="inlineStr">
         <is>
@@ -4761,7 +4739,7 @@
         <v>0.07164</v>
       </c>
       <c r="P13" t="n">
-        <v>0.9120497526158852</v>
+        <v>0.9120497526158851</v>
       </c>
       <c r="Q13" t="inlineStr">
         <is>
@@ -4971,7 +4949,7 @@
         <v>0.8644799999999999</v>
       </c>
       <c r="P16" t="n">
-        <v>0.9768378262820739</v>
+        <v>0.9768378262820741</v>
       </c>
       <c r="Q16" t="inlineStr">
         <is>
@@ -5111,7 +5089,7 @@
         <v>0.31103</v>
       </c>
       <c r="P18" t="n">
-        <v>0.9804206441204166</v>
+        <v>0.9804206441204165</v>
       </c>
       <c r="Q18" t="inlineStr">
         <is>
@@ -5531,7 +5509,7 @@
         <v>0.57823</v>
       </c>
       <c r="P24" t="n">
-        <v>0.9405288652176459</v>
+        <v>0.940528865217646</v>
       </c>
       <c r="Q24" t="inlineStr">
         <is>
@@ -6161,7 +6139,7 @@
         <v>0.75654</v>
       </c>
       <c r="P33" t="n">
-        <v>0.9804206441204166</v>
+        <v>0.9804206441204165</v>
       </c>
       <c r="Q33" t="inlineStr">
         <is>
@@ -6511,7 +6489,7 @@
         <v>0.03781</v>
       </c>
       <c r="P38" t="n">
-        <v>0.9768378262820739</v>
+        <v>0.9768378262820741</v>
       </c>
       <c r="Q38" t="inlineStr">
         <is>
@@ -6791,7 +6769,7 @@
         <v>0.1078</v>
       </c>
       <c r="P42" t="n">
-        <v>0.9258381029412774</v>
+        <v>0.9258381029412773</v>
       </c>
       <c r="Q42" t="inlineStr">
         <is>
@@ -7001,7 +6979,7 @@
         <v>0.20062</v>
       </c>
       <c r="P45" t="n">
-        <v>0.902015239908958</v>
+        <v>0.9020152399089579</v>
       </c>
       <c r="Q45" t="inlineStr">
         <is>
@@ -7141,7 +7119,7 @@
         <v>0.13779</v>
       </c>
       <c r="P47" t="n">
-        <v>0.9120497526158852</v>
+        <v>0.9120497526158851</v>
       </c>
       <c r="Q47" t="inlineStr">
         <is>
@@ -7491,7 +7469,7 @@
         <v>0.43181</v>
       </c>
       <c r="P52" t="n">
-        <v>0.9396635379999008</v>
+        <v>0.9396635379999009</v>
       </c>
       <c r="Q52" t="inlineStr">
         <is>
@@ -7561,7 +7539,7 @@
         <v>0.39722</v>
       </c>
       <c r="P53" t="n">
-        <v>0.972165506193017</v>
+        <v>0.9721655061930171</v>
       </c>
       <c r="Q53" t="inlineStr">
         <is>
@@ -8121,7 +8099,7 @@
         <v>0.24677</v>
       </c>
       <c r="P61" t="n">
-        <v>0.9468448296838138</v>
+        <v>0.9468448296838137</v>
       </c>
       <c r="Q61" t="inlineStr">
         <is>
@@ -8261,7 +8239,7 @@
         <v>0.86456</v>
       </c>
       <c r="P63" t="n">
-        <v>0.9768378262820739</v>
+        <v>0.9768378262820741</v>
       </c>
       <c r="Q63" t="inlineStr">
         <is>
@@ -8401,7 +8379,7 @@
         <v>0.31084</v>
       </c>
       <c r="P65" t="n">
-        <v>0.9804206441204166</v>
+        <v>0.9804206441204165</v>
       </c>
       <c r="Q65" t="inlineStr">
         <is>
@@ -8821,7 +8799,7 @@
         <v>0.57787</v>
       </c>
       <c r="P71" t="n">
-        <v>0.9405288652176459</v>
+        <v>0.940528865217646</v>
       </c>
       <c r="Q71" t="inlineStr">
         <is>
@@ -9521,7 +9499,7 @@
         <v>0.6789799999999999</v>
       </c>
       <c r="P81" t="n">
-        <v>0.972165506193017</v>
+        <v>0.9721655061930171</v>
       </c>
       <c r="Q81" t="inlineStr">
         <is>
@@ -9661,7 +9639,7 @@
         <v>0.41823</v>
       </c>
       <c r="P83" t="n">
-        <v>0.9405288652176459</v>
+        <v>0.940528865217646</v>
       </c>
       <c r="Q83" t="inlineStr">
         <is>
@@ -10711,7 +10689,7 @@
         <v>0.3457</v>
       </c>
       <c r="P98" t="n">
-        <v>0.972165506193017</v>
+        <v>0.9721655061930171</v>
       </c>
       <c r="Q98" t="inlineStr">
         <is>
@@ -10921,7 +10899,7 @@
         <v>0.42233</v>
       </c>
       <c r="P101" t="n">
-        <v>0.9266133026058296</v>
+        <v>0.9266133026058295</v>
       </c>
       <c r="Q101" t="inlineStr">
         <is>
@@ -11481,7 +11459,7 @@
         <v>0.48154</v>
       </c>
       <c r="P109" t="n">
-        <v>0.972165506193017</v>
+        <v>0.9721655061930171</v>
       </c>
       <c r="Q109" t="inlineStr">
         <is>
@@ -11691,7 +11669,7 @@
         <v>0.15134</v>
       </c>
       <c r="P112" t="n">
-        <v>0.9804206441204166</v>
+        <v>0.9804206441204165</v>
       </c>
       <c r="Q112" t="inlineStr">
         <is>
@@ -11901,7 +11879,7 @@
         <v>0.33359</v>
       </c>
       <c r="P115" t="n">
-        <v>0.9266133026058296</v>
+        <v>0.9266133026058295</v>
       </c>
       <c r="Q115" t="inlineStr">
         <is>
@@ -12041,7 +12019,7 @@
         <v>0.1803</v>
       </c>
       <c r="P117" t="n">
-        <v>0.902015239908958</v>
+        <v>0.9020152399089579</v>
       </c>
       <c r="Q117" t="inlineStr">
         <is>
@@ -12181,7 +12159,7 @@
         <v>0.62197</v>
       </c>
       <c r="P119" t="n">
-        <v>0.9266133026058296</v>
+        <v>0.9266133026058295</v>
       </c>
       <c r="Q119" t="inlineStr">
         <is>
@@ -12461,7 +12439,7 @@
         <v>0.37911</v>
       </c>
       <c r="P123" t="n">
-        <v>0.9956462462962075</v>
+        <v>0.9956462462962076</v>
       </c>
       <c r="Q123" t="inlineStr">
         <is>
@@ -12811,7 +12789,7 @@
         <v>0.29213</v>
       </c>
       <c r="P128" t="n">
-        <v>0.972165506193017</v>
+        <v>0.9721655061930171</v>
       </c>
       <c r="Q128" t="inlineStr">
         <is>
@@ -12951,7 +12929,7 @@
         <v>1</v>
       </c>
       <c r="P130" t="n">
-        <v>0.9980786779305384</v>
+        <v>0.9980786779305382</v>
       </c>
       <c r="Q130" t="inlineStr">
         <is>
@@ -13231,7 +13209,7 @@
         <v>0.44641</v>
       </c>
       <c r="P134" t="n">
-        <v>0.9405288652176459</v>
+        <v>0.940528865217646</v>
       </c>
       <c r="Q134" t="inlineStr">
         <is>
@@ -13441,7 +13419,7 @@
         <v>0.20416</v>
       </c>
       <c r="P137" t="n">
-        <v>0.9804206441204166</v>
+        <v>0.9804206441204165</v>
       </c>
       <c r="Q137" t="inlineStr">
         <is>
@@ -13861,7 +13839,7 @@
         <v>0.30868</v>
       </c>
       <c r="P143" t="n">
-        <v>0.902015239908958</v>
+        <v>0.9020152399089579</v>
       </c>
       <c r="Q143" t="inlineStr">
         <is>
@@ -14001,7 +13979,7 @@
         <v>0.07164</v>
       </c>
       <c r="P145" t="n">
-        <v>0.9120497526158852</v>
+        <v>0.9120497526158851</v>
       </c>
       <c r="Q145" t="inlineStr">
         <is>

</xml_diff>